<commit_message>
feat(quotes): lượt 7 — nhập Excel báo giá: cột SL/MOQ + CK %, chọn SP tại chỗ cho dòng mơ hồ, kiểm trùng theo mã khách trước khi tạo SP tạm, file gốc gắn vào báo giá, màn kiểu ERP (07/10)
- lib/quote-excel: qty + discount_pct (tiêu đề VN/EN, không nhầm "SL / thùng"; chặn SL ≤ 0, CK ngoài 0–100) — +4 test
- lib/quote-import-match: candidates cho dòng khớp nhiều SP — +2 test
- quote-import.service: dùng lại SP cùng mã khách của chính khách đó thay vì tạo TMP; SP tạm gắn customer_id; dòng nhận qty/discount; gắn file Excel nguồn vào BG (filesService.attachOrphanToDocument / filesRepo.attachToParent)
- sales/quotes/import: useImportQuote + ImportQuoteScreen (ô đếm là bộ lọc, ProductSearchDialog, thanh chốt đáy bấm được)
- Mẫu Excel sinh lại 22 cột (SL / MOQ, CK %)

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/mau/MAU_BAO_GIA_SP_MOI.xlsx
+++ b/docs/mau/MAU_BAO_GIA_SP_MOI.xlsx
@@ -53,12 +53,26 @@
         </r>
       </text>
     </comment>
+    <comment ref="S3" authorId="0">
+      <text>
+        <r>
+          <t>Số lượng dự kiến hoặc MOQ — bỏ trống nếu chỉ chào đơn giá. In lên tờ báo giá.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="U3" authorId="0">
+      <text>
+        <r>
+          <t>Chiết khấu dòng 0–100, bỏ trống = 0.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="55">
   <si>
     <t>BÁO GIÁ — SẢN PHẨM MỚI</t>
   </si>
@@ -120,9 +134,15 @@
     <t>ĐVT</t>
   </si>
   <si>
+    <t>SL / MOQ</t>
+  </si>
+  <si>
     <t>Đơn giá (FOB) *</t>
   </si>
   <si>
+    <t>CK %</t>
+  </si>
+  <si>
     <t>Ghi chú</t>
   </si>
   <si>
@@ -181,6 +201,9 @@
   </si>
   <si>
     <t>2. Cột có dấu * là bắt buộc: Tên SP, ba số kích thước, Đơn giá.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   SL / MOQ và CK % là tuỳ chọn (07/10/2026): có SL thì tờ in thêm cột Qty + Amount.</t>
   </si>
   <si>
     <t>3. KÍCH THƯỚC — theo đúng bảng kê quy cách của công ty:</t>
@@ -657,7 +680,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T33"/>
+  <dimension ref="A1:V33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -675,11 +698,13 @@
     <col min="14" max="14" width="14" customWidth="1"/>
     <col min="15" max="16" width="10" customWidth="1"/>
     <col min="17" max="17" width="13" customWidth="1"/>
-    <col min="19" max="19" width="14" customWidth="1"/>
-    <col min="20" max="20" width="26" customWidth="1"/>
+    <col min="19" max="19" width="10" customWidth="1"/>
+    <col min="20" max="20" width="14" customWidth="1"/>
+    <col min="21" max="21" width="8" customWidth="1"/>
+    <col min="22" max="22" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -702,8 +727,10 @@
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
-    </row>
-    <row r="2" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+    </row>
+    <row r="2" ht="28" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -726,8 +753,10 @@
       <c r="R2" s="2"/>
       <c r="S2" s="2"/>
       <c r="T2" s="2"/>
-    </row>
-    <row r="3" ht="34" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U2" s="2"/>
+      <c r="V2" s="2"/>
+    </row>
+    <row r="3" ht="34" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -788,8 +817,14 @@
       <c r="T3" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="4" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="V3" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -810,8 +845,10 @@
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
       <c r="T4" s="4"/>
-    </row>
-    <row r="5" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U4" s="4"/>
+      <c r="V4" s="4"/>
+    </row>
+    <row r="5" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -832,8 +869,10 @@
       <c r="R5" s="4"/>
       <c r="S5" s="4"/>
       <c r="T5" s="4"/>
-    </row>
-    <row r="6" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U5" s="4"/>
+      <c r="V5" s="4"/>
+    </row>
+    <row r="6" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="4"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -854,8 +893,10 @@
       <c r="R6" s="4"/>
       <c r="S6" s="4"/>
       <c r="T6" s="4"/>
-    </row>
-    <row r="7" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U6" s="4"/>
+      <c r="V6" s="4"/>
+    </row>
+    <row r="7" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -876,8 +917,10 @@
       <c r="R7" s="4"/>
       <c r="S7" s="4"/>
       <c r="T7" s="4"/>
-    </row>
-    <row r="8" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U7" s="4"/>
+      <c r="V7" s="4"/>
+    </row>
+    <row r="8" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -898,8 +941,10 @@
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
       <c r="T8" s="4"/>
-    </row>
-    <row r="9" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U8" s="4"/>
+      <c r="V8" s="4"/>
+    </row>
+    <row r="9" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -920,8 +965,10 @@
       <c r="R9" s="4"/>
       <c r="S9" s="4"/>
       <c r="T9" s="4"/>
-    </row>
-    <row r="10" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U9" s="4"/>
+      <c r="V9" s="4"/>
+    </row>
+    <row r="10" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -942,8 +989,10 @@
       <c r="R10" s="4"/>
       <c r="S10" s="4"/>
       <c r="T10" s="4"/>
-    </row>
-    <row r="11" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U10" s="4"/>
+      <c r="V10" s="4"/>
+    </row>
+    <row r="11" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -964,8 +1013,10 @@
       <c r="R11" s="4"/>
       <c r="S11" s="4"/>
       <c r="T11" s="4"/>
-    </row>
-    <row r="12" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U11" s="4"/>
+      <c r="V11" s="4"/>
+    </row>
+    <row r="12" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -986,8 +1037,10 @@
       <c r="R12" s="4"/>
       <c r="S12" s="4"/>
       <c r="T12" s="4"/>
-    </row>
-    <row r="13" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U12" s="4"/>
+      <c r="V12" s="4"/>
+    </row>
+    <row r="13" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -1008,8 +1061,10 @@
       <c r="R13" s="4"/>
       <c r="S13" s="4"/>
       <c r="T13" s="4"/>
-    </row>
-    <row r="14" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U13" s="4"/>
+      <c r="V13" s="4"/>
+    </row>
+    <row r="14" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -1030,8 +1085,10 @@
       <c r="R14" s="4"/>
       <c r="S14" s="4"/>
       <c r="T14" s="4"/>
-    </row>
-    <row r="15" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U14" s="4"/>
+      <c r="V14" s="4"/>
+    </row>
+    <row r="15" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -1052,8 +1109,10 @@
       <c r="R15" s="4"/>
       <c r="S15" s="4"/>
       <c r="T15" s="4"/>
-    </row>
-    <row r="16" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U15" s="4"/>
+      <c r="V15" s="4"/>
+    </row>
+    <row r="16" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -1074,8 +1133,10 @@
       <c r="R16" s="4"/>
       <c r="S16" s="4"/>
       <c r="T16" s="4"/>
-    </row>
-    <row r="17" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U16" s="4"/>
+      <c r="V16" s="4"/>
+    </row>
+    <row r="17" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -1096,8 +1157,10 @@
       <c r="R17" s="4"/>
       <c r="S17" s="4"/>
       <c r="T17" s="4"/>
-    </row>
-    <row r="18" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U17" s="4"/>
+      <c r="V17" s="4"/>
+    </row>
+    <row r="18" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A18" s="4"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -1118,8 +1181,10 @@
       <c r="R18" s="4"/>
       <c r="S18" s="4"/>
       <c r="T18" s="4"/>
-    </row>
-    <row r="19" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U18" s="4"/>
+      <c r="V18" s="4"/>
+    </row>
+    <row r="19" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19" s="4"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -1140,8 +1205,10 @@
       <c r="R19" s="4"/>
       <c r="S19" s="4"/>
       <c r="T19" s="4"/>
-    </row>
-    <row r="20" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U19" s="4"/>
+      <c r="V19" s="4"/>
+    </row>
+    <row r="20" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A20" s="4"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -1162,8 +1229,10 @@
       <c r="R20" s="4"/>
       <c r="S20" s="4"/>
       <c r="T20" s="4"/>
-    </row>
-    <row r="21" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U20" s="4"/>
+      <c r="V20" s="4"/>
+    </row>
+    <row r="21" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A21" s="4"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -1184,8 +1253,10 @@
       <c r="R21" s="4"/>
       <c r="S21" s="4"/>
       <c r="T21" s="4"/>
-    </row>
-    <row r="22" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U21" s="4"/>
+      <c r="V21" s="4"/>
+    </row>
+    <row r="22" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22" s="4"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -1206,8 +1277,10 @@
       <c r="R22" s="4"/>
       <c r="S22" s="4"/>
       <c r="T22" s="4"/>
-    </row>
-    <row r="23" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U22" s="4"/>
+      <c r="V22" s="4"/>
+    </row>
+    <row r="23" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A23" s="4"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -1228,8 +1301,10 @@
       <c r="R23" s="4"/>
       <c r="S23" s="4"/>
       <c r="T23" s="4"/>
-    </row>
-    <row r="24" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U23" s="4"/>
+      <c r="V23" s="4"/>
+    </row>
+    <row r="24" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A24" s="4"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -1250,8 +1325,10 @@
       <c r="R24" s="4"/>
       <c r="S24" s="4"/>
       <c r="T24" s="4"/>
-    </row>
-    <row r="25" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U24" s="4"/>
+      <c r="V24" s="4"/>
+    </row>
+    <row r="25" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A25" s="4"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -1272,8 +1349,10 @@
       <c r="R25" s="4"/>
       <c r="S25" s="4"/>
       <c r="T25" s="4"/>
-    </row>
-    <row r="26" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U25" s="4"/>
+      <c r="V25" s="4"/>
+    </row>
+    <row r="26" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A26" s="4"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -1294,8 +1373,10 @@
       <c r="R26" s="4"/>
       <c r="S26" s="4"/>
       <c r="T26" s="4"/>
-    </row>
-    <row r="27" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U26" s="4"/>
+      <c r="V26" s="4"/>
+    </row>
+    <row r="27" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A27" s="4"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -1316,8 +1397,10 @@
       <c r="R27" s="4"/>
       <c r="S27" s="4"/>
       <c r="T27" s="4"/>
-    </row>
-    <row r="28" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U27" s="4"/>
+      <c r="V27" s="4"/>
+    </row>
+    <row r="28" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A28" s="4"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -1338,8 +1421,10 @@
       <c r="R28" s="4"/>
       <c r="S28" s="4"/>
       <c r="T28" s="4"/>
-    </row>
-    <row r="29" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U28" s="4"/>
+      <c r="V28" s="4"/>
+    </row>
+    <row r="29" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -1360,8 +1445,10 @@
       <c r="R29" s="4"/>
       <c r="S29" s="4"/>
       <c r="T29" s="4"/>
-    </row>
-    <row r="30" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U29" s="4"/>
+      <c r="V29" s="4"/>
+    </row>
+    <row r="30" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A30" s="4"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -1382,8 +1469,10 @@
       <c r="R30" s="4"/>
       <c r="S30" s="4"/>
       <c r="T30" s="4"/>
-    </row>
-    <row r="31" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U30" s="4"/>
+      <c r="V30" s="4"/>
+    </row>
+    <row r="31" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A31" s="4"/>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -1404,8 +1493,10 @@
       <c r="R31" s="4"/>
       <c r="S31" s="4"/>
       <c r="T31" s="4"/>
-    </row>
-    <row r="32" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U31" s="4"/>
+      <c r="V31" s="4"/>
+    </row>
+    <row r="32" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A32" s="4"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -1426,8 +1517,10 @@
       <c r="R32" s="4"/>
       <c r="S32" s="4"/>
       <c r="T32" s="4"/>
-    </row>
-    <row r="33" ht="56" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U32" s="4"/>
+      <c r="V32" s="4"/>
+    </row>
+    <row r="33" ht="56" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A33" s="4"/>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -1448,11 +1541,13 @@
       <c r="R33" s="4"/>
       <c r="S33" s="4"/>
       <c r="T33" s="4"/>
+      <c r="U33" s="4"/>
+      <c r="V33" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="A2:T2"/>
+    <mergeCell ref="A1:V1"/>
+    <mergeCell ref="A2:V2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1462,7 +1557,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:V3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1480,11 +1575,13 @@
     <col min="14" max="14" width="14" customWidth="1"/>
     <col min="15" max="16" width="10" customWidth="1"/>
     <col min="17" max="17" width="13" customWidth="1"/>
-    <col min="19" max="19" width="14" customWidth="1"/>
-    <col min="20" max="20" width="26" customWidth="1"/>
+    <col min="19" max="19" width="10" customWidth="1"/>
+    <col min="20" max="20" width="14" customWidth="1"/>
+    <col min="21" max="21" width="8" customWidth="1"/>
+    <col min="22" max="22" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
@@ -1492,7 +1589,7 @@
         <v>3</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>5</v>
@@ -1501,13 +1598,13 @@
         <v>6</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="I1" s="5" t="s">
         <v>10</v>
@@ -1540,27 +1637,33 @@
         <v>19</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="T1" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="U1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="V1" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F2">
         <v>548</v>
@@ -1572,10 +1675,10 @@
         <v>876</v>
       </c>
       <c r="I2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="K2">
         <v>2</v>
@@ -1599,30 +1702,36 @@
         <v>910</v>
       </c>
       <c r="R2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S2">
+        <v>100</v>
+      </c>
+      <c r="T2">
         <v>45.9</v>
       </c>
-      <c r="T2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U2" t="s">
+        <v>29</v>
+      </c>
+      <c r="V2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" t="s">
         <v>29</v>
       </c>
-      <c r="D3" t="s">
-        <v>27</v>
-      </c>
       <c r="E3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F3">
         <v>548</v>
@@ -1634,40 +1743,46 @@
         <v>876</v>
       </c>
       <c r="I3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K3">
         <v>2</v>
       </c>
       <c r="L3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="N3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="O3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="Q3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="R3" t="s">
-        <v>34</v>
-      </c>
-      <c r="S3">
+        <v>36</v>
+      </c>
+      <c r="S3" t="s">
+        <v>29</v>
+      </c>
+      <c r="T3">
         <v>47.5</v>
       </c>
-      <c r="T3" t="s">
-        <v>37</v>
+      <c r="U3">
+        <v>5</v>
+      </c>
+      <c r="V3" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1678,7 +1793,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -1686,102 +1801,107 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>41</v>
+      <c r="A6" s="7" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>42</v>
+      <c r="A7" s="6" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>27</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
-        <v>51</v>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>